<commit_message>
Reconcile May SCL transactions, fix pyarrow error, and hide sidebar status
</commit_message>
<xml_diff>
--- a/Tach_ChiPhi_PP_BL.xlsx
+++ b/Tach_ChiPhi_PP_BL.xlsx
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="E12" s="38" t="n">
-        <v>948924323</v>
+        <v>919245580</v>
       </c>
       <c r="F12" s="39">
         <f>E12*80.79%</f>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="E12" s="38" t="n">
-        <v>320378418</v>
+        <v>320378409</v>
       </c>
       <c r="F12" s="39">
         <f>E12*80.79%</f>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>78353680</v>
+        <v>78353650</v>
       </c>
       <c r="F14" s="39">
         <f>E14*80.79%</f>
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>672123831</v>
+        <v>672123825</v>
       </c>
       <c r="F14" s="39">
         <f>E14*80.79%</f>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E15" s="38" t="n">
-        <v>31618876</v>
+        <v>38379584</v>
       </c>
       <c r="F15" s="39">
         <f>E15*80.79%</f>
@@ -2124,7 +2124,7 @@
         </is>
       </c>
       <c r="E16" s="38" t="n">
-        <v>64930258</v>
+        <v>64792258</v>
       </c>
       <c r="F16" s="39">
         <f>E16*80.79%</f>

</xml_diff>

<commit_message>
Include VTDA in SCL filters to reconcile imports perfectly and match PM_092 SCL net costs
</commit_message>
<xml_diff>
--- a/Tach_ChiPhi_PP_BL.xlsx
+++ b/Tach_ChiPhi_PP_BL.xlsx
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>672123825</v>
+        <v>672123823</v>
       </c>
       <c r="F14" s="39">
         <f>E14*80.79%</f>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E15" s="38" t="n">
-        <v>38379584</v>
+        <v>38379478</v>
       </c>
       <c r="F15" s="39">
         <f>E15*80.79%</f>

</xml_diff>